<commit_message>
update the output of visits
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Output_visits_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/Output_visits_Raw.xlsx
@@ -504,7 +504,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>14.11</v>
+        <v>7.06</v>
       </c>
       <c r="C3">
         <v>0.5</v>
@@ -652,25 +652,25 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>30.7</v>
+        <v>16.15</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>426</v>
+        <v>298</v>
       </c>
       <c r="E2">
-        <v>24.03</v>
+        <v>14.33</v>
       </c>
       <c r="F2">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="G2">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H2">
-        <v>39</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -678,25 +678,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>24.23</v>
+        <v>6.84</v>
       </c>
       <c r="C3">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>166</v>
+        <v>95.5</v>
       </c>
       <c r="E3">
-        <v>11.08</v>
+        <v>6.54</v>
       </c>
       <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>2.5</v>
+      </c>
+      <c r="H3">
         <v>9</v>
-      </c>
-      <c r="G3">
-        <v>4.5</v>
-      </c>
-      <c r="H3">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>